<commit_message>
Travaux du 01/10/2026 matin
</commit_message>
<xml_diff>
--- a/public/Recuperation heures pour export.xlsx
+++ b/public/Recuperation heures pour export.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\zoul\Documents\POLYNOV\polynov-temps\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{65C6670E-C315-4F7B-9F3E-68E3EA90399A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E58DF0C-F2C7-42A0-8350-3C803E1B9FEB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="788" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1564,30 +1564,6 @@
     <xf numFmtId="0" fontId="11" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="8" borderId="7" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="8" borderId="5" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="2" borderId="7" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1618,10 +1594,46 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="0" fillId="8" borderId="7" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="8" borderId="5" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="2" borderId="7" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1630,31 +1642,19 @@
     <xf numFmtId="0" fontId="11" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -2610,7 +2610,7 @@
   <dimension ref="A1:BC2"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="15.44140625" style="9" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="20.77734375" style="9" customWidth="1"/>
     <col min="2" max="2" width="6" style="5" customWidth="1"/>
     <col min="3" max="3" width="11.88671875" style="6" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="10.44140625" style="8" bestFit="1" customWidth="1"/>
@@ -2624,100 +2624,100 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:55" ht="49.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="50" t="s">
+      <c r="A1" s="42" t="s">
         <v>27</v>
       </c>
       <c r="B1" s="17"/>
-      <c r="C1" s="52" t="s">
+      <c r="C1" s="44" t="s">
         <v>28</v>
       </c>
-      <c r="D1" s="54" t="s">
+      <c r="D1" s="46" t="s">
         <v>29</v>
       </c>
-      <c r="E1" s="56" t="s">
+      <c r="E1" s="48" t="s">
         <v>14</v>
       </c>
-      <c r="F1" s="56"/>
-      <c r="G1" s="56"/>
-      <c r="H1" s="56"/>
-      <c r="I1" s="56"/>
-      <c r="J1" s="56"/>
-      <c r="K1" s="56"/>
-      <c r="L1" s="56"/>
-      <c r="M1" s="56"/>
-      <c r="N1" s="56"/>
-      <c r="O1" s="56"/>
-      <c r="P1" s="56"/>
-      <c r="Q1" s="56"/>
-      <c r="R1" s="56"/>
-      <c r="S1" s="56"/>
-      <c r="T1" s="56"/>
-      <c r="U1" s="56"/>
-      <c r="V1" s="56"/>
-      <c r="W1" s="56"/>
-      <c r="X1" s="56"/>
-      <c r="Y1" s="56"/>
-      <c r="Z1" s="57" t="s">
+      <c r="F1" s="48"/>
+      <c r="G1" s="48"/>
+      <c r="H1" s="48"/>
+      <c r="I1" s="48"/>
+      <c r="J1" s="48"/>
+      <c r="K1" s="48"/>
+      <c r="L1" s="48"/>
+      <c r="M1" s="48"/>
+      <c r="N1" s="48"/>
+      <c r="O1" s="48"/>
+      <c r="P1" s="48"/>
+      <c r="Q1" s="48"/>
+      <c r="R1" s="48"/>
+      <c r="S1" s="48"/>
+      <c r="T1" s="48"/>
+      <c r="U1" s="48"/>
+      <c r="V1" s="48"/>
+      <c r="W1" s="48"/>
+      <c r="X1" s="48"/>
+      <c r="Y1" s="48"/>
+      <c r="Z1" s="49" t="s">
         <v>24</v>
       </c>
-      <c r="AA1" s="58"/>
-      <c r="AB1" s="58"/>
-      <c r="AC1" s="58"/>
-      <c r="AD1" s="58"/>
-      <c r="AE1" s="58"/>
-      <c r="AF1" s="58"/>
-      <c r="AG1" s="58"/>
-      <c r="AH1" s="58"/>
-      <c r="AI1" s="58"/>
-      <c r="AJ1" s="58"/>
-      <c r="AK1" s="58"/>
-      <c r="AL1" s="58"/>
-      <c r="AM1" s="58"/>
-      <c r="AN1" s="58"/>
-      <c r="AO1" s="59"/>
-      <c r="AP1" s="44" t="e">
+      <c r="AA1" s="50"/>
+      <c r="AB1" s="50"/>
+      <c r="AC1" s="50"/>
+      <c r="AD1" s="50"/>
+      <c r="AE1" s="50"/>
+      <c r="AF1" s="50"/>
+      <c r="AG1" s="50"/>
+      <c r="AH1" s="50"/>
+      <c r="AI1" s="50"/>
+      <c r="AJ1" s="50"/>
+      <c r="AK1" s="50"/>
+      <c r="AL1" s="50"/>
+      <c r="AM1" s="50"/>
+      <c r="AN1" s="50"/>
+      <c r="AO1" s="51"/>
+      <c r="AP1" s="54" t="e">
         <f>"LUNDI" &amp; CHAR(10) &amp; TEXT(7*B2+DATE(B1,1,3)-WEEKDAY(DATE(B1,1,3))-5,"JJ/MM/AA")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="AQ1" s="45"/>
-      <c r="AR1" s="46" t="e">
+      <c r="AQ1" s="55"/>
+      <c r="AR1" s="56" t="e">
         <f>"MARDI" &amp; CHAR(10) &amp; TEXT(7*B2+DATE(B1,1,3)-WEEKDAY(DATE(B1,1,3))-4,"JJ/MM/AA")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="AS1" s="47"/>
-      <c r="AT1" s="48" t="e">
+      <c r="AS1" s="57"/>
+      <c r="AT1" s="58" t="e">
         <f>"MERCREDI" &amp; CHAR(10) &amp; TEXT(7*B2+DATE(B1,1,3)-WEEKDAY(DATE(B1,1,3))-3,"JJ/MM/AA")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="AU1" s="49"/>
-      <c r="AV1" s="46" t="e">
+      <c r="AU1" s="59"/>
+      <c r="AV1" s="56" t="e">
         <f>"JEUDI" &amp; CHAR(10) &amp; TEXT(7*B2+DATE(B1,1,3)-WEEKDAY(DATE(B1,1,3))-2,"JJ/MM/AA")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="AW1" s="47"/>
-      <c r="AX1" s="48" t="e">
+      <c r="AW1" s="57"/>
+      <c r="AX1" s="58" t="e">
         <f>"VENDREDI" &amp; CHAR(10) &amp; TEXT(7*B2+DATE(B1,1,3)-WEEKDAY(DATE(B1,1,3))-1,"JJ/MM/AA")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="AY1" s="49"/>
-      <c r="AZ1" s="42" t="str">
+      <c r="AY1" s="59"/>
+      <c r="AZ1" s="52" t="str">
         <f>"SAMEDI" &amp; CHAR(10) &amp; TEXT(7*B2+DATE(B1,1,3)-WEEKDAY(DATE(B1,1,3)),"JJ/MM/AA")</f>
         <v>SAMEDI
 00/01/00</v>
       </c>
-      <c r="BA1" s="43"/>
-      <c r="BB1" s="42" t="str">
+      <c r="BA1" s="53"/>
+      <c r="BB1" s="52" t="str">
         <f>"DIMANCHE" &amp; CHAR(10) &amp; TEXT(7*B2+DATE(B1,1,3)-WEEKDAY(DATE(B1,1,3))+1,"JJ/MM/AA")</f>
         <v>DIMANCHE
 01/01/00</v>
       </c>
-      <c r="BC1" s="43"/>
+      <c r="BC1" s="53"/>
     </row>
     <row r="2" spans="1:55" s="1" customFormat="1" ht="18" x14ac:dyDescent="0.3">
-      <c r="A2" s="51"/>
+      <c r="A2" s="43"/>
       <c r="B2" s="16"/>
-      <c r="C2" s="53"/>
-      <c r="D2" s="55"/>
+      <c r="C2" s="45"/>
+      <c r="D2" s="47"/>
       <c r="E2" s="2"/>
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
@@ -2801,11 +2801,6 @@
   </sheetData>
   <dataConsolidate/>
   <mergeCells count="12">
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="C1:C2"/>
-    <mergeCell ref="D1:D2"/>
-    <mergeCell ref="E1:Y1"/>
-    <mergeCell ref="Z1:AO1"/>
     <mergeCell ref="BB1:BC1"/>
     <mergeCell ref="AP1:AQ1"/>
     <mergeCell ref="AR1:AS1"/>
@@ -2813,6 +2808,11 @@
     <mergeCell ref="AV1:AW1"/>
     <mergeCell ref="AX1:AY1"/>
     <mergeCell ref="AZ1:BA1"/>
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="C1:C2"/>
+    <mergeCell ref="D1:D2"/>
+    <mergeCell ref="E1:Y1"/>
+    <mergeCell ref="Z1:AO1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -2839,109 +2839,109 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:55" ht="49.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="50" t="s">
+      <c r="A1" s="42" t="s">
         <v>27</v>
       </c>
       <c r="B1" s="17" t="s">
         <v>83</v>
       </c>
-      <c r="C1" s="52" t="s">
+      <c r="C1" s="44" t="s">
         <v>28</v>
       </c>
-      <c r="D1" s="54" t="s">
+      <c r="D1" s="46" t="s">
         <v>29</v>
       </c>
-      <c r="E1" s="56" t="s">
+      <c r="E1" s="48" t="s">
         <v>14</v>
       </c>
-      <c r="F1" s="56"/>
-      <c r="G1" s="56"/>
-      <c r="H1" s="56"/>
-      <c r="I1" s="56"/>
-      <c r="J1" s="56"/>
-      <c r="K1" s="56"/>
-      <c r="L1" s="56"/>
-      <c r="M1" s="56"/>
-      <c r="N1" s="56"/>
-      <c r="O1" s="56"/>
-      <c r="P1" s="56"/>
-      <c r="Q1" s="56"/>
-      <c r="R1" s="56"/>
-      <c r="S1" s="56"/>
-      <c r="T1" s="56"/>
-      <c r="U1" s="56"/>
-      <c r="V1" s="56"/>
-      <c r="W1" s="56"/>
-      <c r="X1" s="56"/>
-      <c r="Y1" s="56"/>
-      <c r="Z1" s="57" t="s">
+      <c r="F1" s="48"/>
+      <c r="G1" s="48"/>
+      <c r="H1" s="48"/>
+      <c r="I1" s="48"/>
+      <c r="J1" s="48"/>
+      <c r="K1" s="48"/>
+      <c r="L1" s="48"/>
+      <c r="M1" s="48"/>
+      <c r="N1" s="48"/>
+      <c r="O1" s="48"/>
+      <c r="P1" s="48"/>
+      <c r="Q1" s="48"/>
+      <c r="R1" s="48"/>
+      <c r="S1" s="48"/>
+      <c r="T1" s="48"/>
+      <c r="U1" s="48"/>
+      <c r="V1" s="48"/>
+      <c r="W1" s="48"/>
+      <c r="X1" s="48"/>
+      <c r="Y1" s="48"/>
+      <c r="Z1" s="49" t="s">
         <v>24</v>
       </c>
-      <c r="AA1" s="58"/>
-      <c r="AB1" s="58"/>
-      <c r="AC1" s="58"/>
-      <c r="AD1" s="58"/>
-      <c r="AE1" s="58"/>
-      <c r="AF1" s="58"/>
-      <c r="AG1" s="58"/>
-      <c r="AH1" s="58"/>
-      <c r="AI1" s="58"/>
-      <c r="AJ1" s="58"/>
-      <c r="AK1" s="58"/>
-      <c r="AL1" s="58"/>
-      <c r="AM1" s="58"/>
-      <c r="AN1" s="58"/>
-      <c r="AO1" s="59"/>
-      <c r="AP1" s="44" t="str">
+      <c r="AA1" s="50"/>
+      <c r="AB1" s="50"/>
+      <c r="AC1" s="50"/>
+      <c r="AD1" s="50"/>
+      <c r="AE1" s="50"/>
+      <c r="AF1" s="50"/>
+      <c r="AG1" s="50"/>
+      <c r="AH1" s="50"/>
+      <c r="AI1" s="50"/>
+      <c r="AJ1" s="50"/>
+      <c r="AK1" s="50"/>
+      <c r="AL1" s="50"/>
+      <c r="AM1" s="50"/>
+      <c r="AN1" s="50"/>
+      <c r="AO1" s="51"/>
+      <c r="AP1" s="54" t="str">
         <f>"LUNDI" &amp; CHAR(10) &amp; TEXT(7*B2+DATE(B1,1,3)-WEEKDAY(DATE(B1,1,3))-5,"JJ/MM/AA")</f>
         <v>LUNDI
 21/09/26</v>
       </c>
-      <c r="AQ1" s="45"/>
-      <c r="AR1" s="46" t="str">
+      <c r="AQ1" s="55"/>
+      <c r="AR1" s="56" t="str">
         <f>"MARDI" &amp; CHAR(10) &amp; TEXT(7*B2+DATE(B1,1,3)-WEEKDAY(DATE(B1,1,3))-4,"JJ/MM/AA")</f>
         <v>MARDI
 22/09/26</v>
       </c>
-      <c r="AS1" s="47"/>
-      <c r="AT1" s="48" t="str">
+      <c r="AS1" s="57"/>
+      <c r="AT1" s="58" t="str">
         <f>"MERCREDI" &amp; CHAR(10) &amp; TEXT(7*B2+DATE(B1,1,3)-WEEKDAY(DATE(B1,1,3))-3,"JJ/MM/AA")</f>
         <v>MERCREDI
 23/09/26</v>
       </c>
-      <c r="AU1" s="49"/>
-      <c r="AV1" s="46" t="str">
+      <c r="AU1" s="59"/>
+      <c r="AV1" s="56" t="str">
         <f>"JEUDI" &amp; CHAR(10) &amp; TEXT(7*B2+DATE(B1,1,3)-WEEKDAY(DATE(B1,1,3))-2,"JJ/MM/AA")</f>
         <v>JEUDI
 24/09/26</v>
       </c>
-      <c r="AW1" s="47"/>
-      <c r="AX1" s="48" t="str">
+      <c r="AW1" s="57"/>
+      <c r="AX1" s="58" t="str">
         <f>"VENDREDI" &amp; CHAR(10) &amp; TEXT(7*B2+DATE(B1,1,3)-WEEKDAY(DATE(B1,1,3))-1,"JJ/MM/AA")</f>
         <v>VENDREDI
 25/09/26</v>
       </c>
-      <c r="AY1" s="49"/>
-      <c r="AZ1" s="42" t="str">
+      <c r="AY1" s="59"/>
+      <c r="AZ1" s="52" t="str">
         <f>"SAMEDI" &amp; CHAR(10) &amp; TEXT(7*B2+DATE(B1,1,3)-WEEKDAY(DATE(B1,1,3)),"JJ/MM/AA")</f>
         <v>SAMEDI
 26/09/26</v>
       </c>
-      <c r="BA1" s="43"/>
-      <c r="BB1" s="42" t="str">
+      <c r="BA1" s="53"/>
+      <c r="BB1" s="52" t="str">
         <f>"DIMANCHE" &amp; CHAR(10) &amp; TEXT(7*B2+DATE(B1,1,3)-WEEKDAY(DATE(B1,1,3))+1,"JJ/MM/AA")</f>
         <v>DIMANCHE
 27/09/26</v>
       </c>
-      <c r="BC1" s="43"/>
+      <c r="BC1" s="53"/>
     </row>
     <row r="2" spans="1:55" s="1" customFormat="1" ht="18" x14ac:dyDescent="0.3">
-      <c r="A2" s="51"/>
+      <c r="A2" s="43"/>
       <c r="B2" s="16" t="s">
         <v>42</v>
       </c>
-      <c r="C2" s="53"/>
-      <c r="D2" s="55"/>
+      <c r="C2" s="45"/>
+      <c r="D2" s="47"/>
       <c r="E2" s="2" t="s">
         <v>0</v>
       </c>
@@ -3200,26 +3200,26 @@
       <c r="AM8" s="28"/>
       <c r="AN8" s="28"/>
       <c r="AO8" s="28"/>
-      <c r="AP8" s="62">
+      <c r="AP8" s="66">
         <v>7.5</v>
       </c>
-      <c r="AQ8" s="63"/>
-      <c r="AR8" s="64">
+      <c r="AQ8" s="67"/>
+      <c r="AR8" s="62">
         <v>7.5</v>
       </c>
-      <c r="AS8" s="65"/>
-      <c r="AT8" s="62">
+      <c r="AS8" s="63"/>
+      <c r="AT8" s="66">
         <v>7.5</v>
       </c>
-      <c r="AU8" s="63"/>
-      <c r="AV8" s="64">
+      <c r="AU8" s="67"/>
+      <c r="AV8" s="62">
         <v>7.5</v>
       </c>
-      <c r="AW8" s="65"/>
-      <c r="AX8" s="62">
+      <c r="AW8" s="63"/>
+      <c r="AX8" s="66">
         <v>5</v>
       </c>
-      <c r="AY8" s="63"/>
+      <c r="AY8" s="67"/>
       <c r="AZ8" s="29">
         <v>0</v>
       </c>
@@ -3351,26 +3351,26 @@
       <c r="AM10" s="23"/>
       <c r="AN10" s="23"/>
       <c r="AO10" s="32"/>
-      <c r="AP10" s="66" t="s">
+      <c r="AP10" s="60" t="s">
         <v>46</v>
       </c>
-      <c r="AQ10" s="67"/>
-      <c r="AR10" s="66" t="s">
+      <c r="AQ10" s="61"/>
+      <c r="AR10" s="60" t="s">
         <v>46</v>
       </c>
-      <c r="AS10" s="67"/>
-      <c r="AT10" s="66" t="s">
+      <c r="AS10" s="61"/>
+      <c r="AT10" s="60" t="s">
         <v>46</v>
       </c>
-      <c r="AU10" s="67"/>
-      <c r="AV10" s="66" t="s">
+      <c r="AU10" s="61"/>
+      <c r="AV10" s="60" t="s">
         <v>46</v>
       </c>
-      <c r="AW10" s="67"/>
-      <c r="AX10" s="70" t="s">
+      <c r="AW10" s="61"/>
+      <c r="AX10" s="64" t="s">
         <v>45</v>
       </c>
-      <c r="AY10" s="72"/>
+      <c r="AY10" s="65"/>
       <c r="AZ10" s="33"/>
       <c r="BA10" s="24"/>
       <c r="BB10" s="24"/>
@@ -3496,26 +3496,26 @@
       <c r="AM17" s="28"/>
       <c r="AN17" s="28"/>
       <c r="AO17" s="28"/>
-      <c r="AP17" s="62">
+      <c r="AP17" s="66">
         <v>7.5</v>
       </c>
-      <c r="AQ17" s="63"/>
-      <c r="AR17" s="64">
+      <c r="AQ17" s="67"/>
+      <c r="AR17" s="62">
         <v>7.5</v>
       </c>
-      <c r="AS17" s="65"/>
-      <c r="AT17" s="62">
+      <c r="AS17" s="63"/>
+      <c r="AT17" s="66">
         <v>7.5</v>
       </c>
-      <c r="AU17" s="63"/>
-      <c r="AV17" s="64">
+      <c r="AU17" s="67"/>
+      <c r="AV17" s="62">
         <v>7.5</v>
       </c>
-      <c r="AW17" s="65"/>
-      <c r="AX17" s="62">
+      <c r="AW17" s="63"/>
+      <c r="AX17" s="66">
         <v>5</v>
       </c>
-      <c r="AY17" s="63"/>
+      <c r="AY17" s="67"/>
       <c r="AZ17" s="29">
         <v>0</v>
       </c>
@@ -3647,23 +3647,23 @@
       <c r="AM19" s="23"/>
       <c r="AN19" s="23"/>
       <c r="AO19" s="32"/>
-      <c r="AP19" s="66" t="s">
+      <c r="AP19" s="60" t="s">
         <v>46</v>
       </c>
-      <c r="AQ19" s="67"/>
-      <c r="AR19" s="66" t="s">
+      <c r="AQ19" s="61"/>
+      <c r="AR19" s="60" t="s">
         <v>46</v>
       </c>
-      <c r="AS19" s="67"/>
-      <c r="AT19" s="66" t="s">
+      <c r="AS19" s="61"/>
+      <c r="AT19" s="60" t="s">
         <v>46</v>
       </c>
-      <c r="AU19" s="67"/>
-      <c r="AV19" s="66" t="s">
+      <c r="AU19" s="61"/>
+      <c r="AV19" s="60" t="s">
         <v>46</v>
       </c>
-      <c r="AW19" s="67"/>
-      <c r="AX19" s="66" t="s">
+      <c r="AW19" s="61"/>
+      <c r="AX19" s="60" t="s">
         <v>46</v>
       </c>
       <c r="AY19" s="68"/>
@@ -3743,26 +3743,26 @@
       <c r="AM23" s="28"/>
       <c r="AN23" s="28"/>
       <c r="AO23" s="28"/>
-      <c r="AP23" s="62">
+      <c r="AP23" s="66">
         <v>7.5</v>
       </c>
-      <c r="AQ23" s="63"/>
-      <c r="AR23" s="64">
+      <c r="AQ23" s="67"/>
+      <c r="AR23" s="62">
         <v>7.5</v>
       </c>
-      <c r="AS23" s="65"/>
-      <c r="AT23" s="62">
+      <c r="AS23" s="63"/>
+      <c r="AT23" s="66">
         <v>7.5</v>
       </c>
-      <c r="AU23" s="63"/>
-      <c r="AV23" s="64">
+      <c r="AU23" s="67"/>
+      <c r="AV23" s="62">
         <v>7.5</v>
       </c>
-      <c r="AW23" s="65"/>
-      <c r="AX23" s="62">
+      <c r="AW23" s="63"/>
+      <c r="AX23" s="66">
         <v>5</v>
       </c>
-      <c r="AY23" s="63"/>
+      <c r="AY23" s="67"/>
       <c r="AZ23" s="29">
         <v>0</v>
       </c>
@@ -3894,23 +3894,23 @@
       <c r="AM25" s="23"/>
       <c r="AN25" s="23"/>
       <c r="AO25" s="32"/>
-      <c r="AP25" s="66" t="s">
+      <c r="AP25" s="60" t="s">
         <v>46</v>
       </c>
-      <c r="AQ25" s="67"/>
-      <c r="AR25" s="66" t="s">
+      <c r="AQ25" s="61"/>
+      <c r="AR25" s="60" t="s">
         <v>46</v>
       </c>
-      <c r="AS25" s="67"/>
-      <c r="AT25" s="66" t="s">
+      <c r="AS25" s="61"/>
+      <c r="AT25" s="60" t="s">
         <v>46</v>
       </c>
-      <c r="AU25" s="67"/>
-      <c r="AV25" s="66" t="s">
+      <c r="AU25" s="61"/>
+      <c r="AV25" s="60" t="s">
         <v>46</v>
       </c>
-      <c r="AW25" s="67"/>
-      <c r="AX25" s="66" t="s">
+      <c r="AW25" s="61"/>
+      <c r="AX25" s="60" t="s">
         <v>46</v>
       </c>
       <c r="AY25" s="68"/>
@@ -3990,26 +3990,26 @@
       <c r="AM29" s="28"/>
       <c r="AN29" s="28"/>
       <c r="AO29" s="28"/>
-      <c r="AP29" s="62">
+      <c r="AP29" s="66">
         <v>8</v>
       </c>
-      <c r="AQ29" s="63"/>
-      <c r="AR29" s="64">
+      <c r="AQ29" s="67"/>
+      <c r="AR29" s="62">
         <v>8</v>
       </c>
-      <c r="AS29" s="65"/>
-      <c r="AT29" s="62">
+      <c r="AS29" s="63"/>
+      <c r="AT29" s="66">
         <v>8</v>
       </c>
-      <c r="AU29" s="63"/>
-      <c r="AV29" s="64">
+      <c r="AU29" s="67"/>
+      <c r="AV29" s="62">
         <v>8</v>
       </c>
-      <c r="AW29" s="65"/>
-      <c r="AX29" s="62">
+      <c r="AW29" s="63"/>
+      <c r="AX29" s="66">
         <v>5.5</v>
       </c>
-      <c r="AY29" s="63"/>
+      <c r="AY29" s="67"/>
       <c r="AZ29" s="29">
         <v>0</v>
       </c>
@@ -4144,26 +4144,26 @@
       <c r="AM31" s="23"/>
       <c r="AN31" s="23"/>
       <c r="AO31" s="32"/>
-      <c r="AP31" s="70" t="s">
+      <c r="AP31" s="64" t="s">
         <v>45</v>
       </c>
-      <c r="AQ31" s="71"/>
-      <c r="AR31" s="70" t="s">
+      <c r="AQ31" s="69"/>
+      <c r="AR31" s="64" t="s">
         <v>45</v>
       </c>
-      <c r="AS31" s="71"/>
-      <c r="AT31" s="66" t="s">
+      <c r="AS31" s="69"/>
+      <c r="AT31" s="60" t="s">
         <v>46</v>
       </c>
-      <c r="AU31" s="67"/>
-      <c r="AV31" s="66" t="s">
+      <c r="AU31" s="61"/>
+      <c r="AV31" s="60" t="s">
         <v>46</v>
       </c>
-      <c r="AW31" s="67"/>
-      <c r="AX31" s="70" t="s">
+      <c r="AW31" s="61"/>
+      <c r="AX31" s="64" t="s">
         <v>45</v>
       </c>
-      <c r="AY31" s="72"/>
+      <c r="AY31" s="65"/>
       <c r="AZ31" s="33"/>
       <c r="BA31" s="24"/>
       <c r="BB31" s="24"/>
@@ -4246,26 +4246,26 @@
       <c r="AM35" s="28"/>
       <c r="AN35" s="28"/>
       <c r="AO35" s="28"/>
-      <c r="AP35" s="62">
+      <c r="AP35" s="66">
         <v>7.5</v>
       </c>
-      <c r="AQ35" s="63"/>
-      <c r="AR35" s="64">
+      <c r="AQ35" s="67"/>
+      <c r="AR35" s="62">
         <v>7.5</v>
       </c>
-      <c r="AS35" s="65"/>
-      <c r="AT35" s="62">
+      <c r="AS35" s="63"/>
+      <c r="AT35" s="66">
         <v>7.5</v>
       </c>
-      <c r="AU35" s="63"/>
-      <c r="AV35" s="64">
+      <c r="AU35" s="67"/>
+      <c r="AV35" s="62">
         <v>7.5</v>
       </c>
-      <c r="AW35" s="65"/>
-      <c r="AX35" s="62">
+      <c r="AW35" s="63"/>
+      <c r="AX35" s="66">
         <v>5</v>
       </c>
-      <c r="AY35" s="63"/>
+      <c r="AY35" s="67"/>
       <c r="AZ35" s="29">
         <v>0</v>
       </c>
@@ -4397,23 +4397,23 @@
       <c r="AM37" s="23"/>
       <c r="AN37" s="23"/>
       <c r="AO37" s="32"/>
-      <c r="AP37" s="66" t="s">
+      <c r="AP37" s="60" t="s">
         <v>46</v>
       </c>
-      <c r="AQ37" s="67"/>
-      <c r="AR37" s="66" t="s">
+      <c r="AQ37" s="61"/>
+      <c r="AR37" s="60" t="s">
         <v>46</v>
       </c>
-      <c r="AS37" s="67"/>
-      <c r="AT37" s="66" t="s">
+      <c r="AS37" s="61"/>
+      <c r="AT37" s="60" t="s">
         <v>46</v>
       </c>
-      <c r="AU37" s="67"/>
-      <c r="AV37" s="66" t="s">
+      <c r="AU37" s="61"/>
+      <c r="AV37" s="60" t="s">
         <v>46</v>
       </c>
-      <c r="AW37" s="67"/>
-      <c r="AX37" s="66" t="s">
+      <c r="AW37" s="61"/>
+      <c r="AX37" s="60" t="s">
         <v>46</v>
       </c>
       <c r="AY37" s="68"/>
@@ -4493,26 +4493,26 @@
       <c r="AM41" s="28"/>
       <c r="AN41" s="28"/>
       <c r="AO41" s="28"/>
-      <c r="AP41" s="62">
+      <c r="AP41" s="66">
         <v>7.5</v>
       </c>
-      <c r="AQ41" s="63"/>
-      <c r="AR41" s="64">
+      <c r="AQ41" s="67"/>
+      <c r="AR41" s="62">
         <v>7.5</v>
       </c>
-      <c r="AS41" s="65"/>
-      <c r="AT41" s="62">
+      <c r="AS41" s="63"/>
+      <c r="AT41" s="66">
         <v>7.5</v>
       </c>
-      <c r="AU41" s="63"/>
-      <c r="AV41" s="64">
+      <c r="AU41" s="67"/>
+      <c r="AV41" s="62">
         <v>7.5</v>
       </c>
-      <c r="AW41" s="65"/>
-      <c r="AX41" s="62">
+      <c r="AW41" s="63"/>
+      <c r="AX41" s="66">
         <v>5</v>
       </c>
-      <c r="AY41" s="63"/>
+      <c r="AY41" s="67"/>
       <c r="AZ41" s="29">
         <v>0</v>
       </c>
@@ -4644,23 +4644,23 @@
       <c r="AM43" s="23"/>
       <c r="AN43" s="23"/>
       <c r="AO43" s="32"/>
-      <c r="AP43" s="66" t="s">
+      <c r="AP43" s="60" t="s">
         <v>46</v>
       </c>
-      <c r="AQ43" s="67"/>
-      <c r="AR43" s="66" t="s">
+      <c r="AQ43" s="61"/>
+      <c r="AR43" s="60" t="s">
         <v>46</v>
       </c>
-      <c r="AS43" s="67"/>
-      <c r="AT43" s="66" t="s">
+      <c r="AS43" s="61"/>
+      <c r="AT43" s="60" t="s">
         <v>46</v>
       </c>
-      <c r="AU43" s="67"/>
-      <c r="AV43" s="66" t="s">
+      <c r="AU43" s="61"/>
+      <c r="AV43" s="60" t="s">
         <v>46</v>
       </c>
-      <c r="AW43" s="67"/>
-      <c r="AX43" s="66" t="s">
+      <c r="AW43" s="61"/>
+      <c r="AX43" s="60" t="s">
         <v>46</v>
       </c>
       <c r="AY43" s="68"/>
@@ -4759,26 +4759,26 @@
       <c r="AM48" s="28"/>
       <c r="AN48" s="28"/>
       <c r="AO48" s="28"/>
-      <c r="AP48" s="62">
+      <c r="AP48" s="66">
         <v>7.5</v>
       </c>
-      <c r="AQ48" s="63"/>
-      <c r="AR48" s="64">
+      <c r="AQ48" s="67"/>
+      <c r="AR48" s="62">
         <v>7.5</v>
       </c>
-      <c r="AS48" s="65"/>
-      <c r="AT48" s="62">
+      <c r="AS48" s="63"/>
+      <c r="AT48" s="66">
         <v>7.5</v>
       </c>
-      <c r="AU48" s="63"/>
-      <c r="AV48" s="64">
+      <c r="AU48" s="67"/>
+      <c r="AV48" s="62">
         <v>7.5</v>
       </c>
-      <c r="AW48" s="65"/>
-      <c r="AX48" s="62">
+      <c r="AW48" s="63"/>
+      <c r="AX48" s="66">
         <v>5</v>
       </c>
-      <c r="AY48" s="63"/>
+      <c r="AY48" s="67"/>
       <c r="AZ48" s="29">
         <v>0</v>
       </c>
@@ -4910,23 +4910,23 @@
       <c r="AM50" s="23"/>
       <c r="AN50" s="23"/>
       <c r="AO50" s="32"/>
-      <c r="AP50" s="66" t="s">
+      <c r="AP50" s="60" t="s">
         <v>46</v>
       </c>
-      <c r="AQ50" s="67"/>
-      <c r="AR50" s="66" t="s">
+      <c r="AQ50" s="61"/>
+      <c r="AR50" s="60" t="s">
         <v>46</v>
       </c>
-      <c r="AS50" s="67"/>
-      <c r="AT50" s="66" t="s">
+      <c r="AS50" s="61"/>
+      <c r="AT50" s="60" t="s">
         <v>46</v>
       </c>
-      <c r="AU50" s="67"/>
-      <c r="AV50" s="66" t="s">
+      <c r="AU50" s="61"/>
+      <c r="AV50" s="60" t="s">
         <v>46</v>
       </c>
-      <c r="AW50" s="67"/>
-      <c r="AX50" s="66" t="s">
+      <c r="AW50" s="61"/>
+      <c r="AX50" s="60" t="s">
         <v>46</v>
       </c>
       <c r="AY50" s="68"/>
@@ -5003,26 +5003,26 @@
       <c r="AM54" s="28"/>
       <c r="AN54" s="28"/>
       <c r="AO54" s="28"/>
-      <c r="AP54" s="62">
+      <c r="AP54" s="66">
         <v>7.5</v>
       </c>
-      <c r="AQ54" s="63"/>
-      <c r="AR54" s="64">
+      <c r="AQ54" s="67"/>
+      <c r="AR54" s="62">
         <v>7.5</v>
       </c>
-      <c r="AS54" s="65"/>
-      <c r="AT54" s="62">
+      <c r="AS54" s="63"/>
+      <c r="AT54" s="66">
         <v>7.5</v>
       </c>
-      <c r="AU54" s="63"/>
-      <c r="AV54" s="64">
+      <c r="AU54" s="67"/>
+      <c r="AV54" s="62">
         <v>7.5</v>
       </c>
-      <c r="AW54" s="65"/>
-      <c r="AX54" s="62">
+      <c r="AW54" s="63"/>
+      <c r="AX54" s="66">
         <v>5</v>
       </c>
-      <c r="AY54" s="63"/>
+      <c r="AY54" s="67"/>
       <c r="AZ54" s="29">
         <v>0</v>
       </c>
@@ -5154,23 +5154,23 @@
       <c r="AM56" s="23"/>
       <c r="AN56" s="23"/>
       <c r="AO56" s="32"/>
-      <c r="AP56" s="66" t="s">
+      <c r="AP56" s="60" t="s">
         <v>46</v>
       </c>
-      <c r="AQ56" s="67"/>
-      <c r="AR56" s="66" t="s">
+      <c r="AQ56" s="61"/>
+      <c r="AR56" s="60" t="s">
         <v>46</v>
       </c>
-      <c r="AS56" s="67"/>
-      <c r="AT56" s="66" t="s">
+      <c r="AS56" s="61"/>
+      <c r="AT56" s="60" t="s">
         <v>46</v>
       </c>
-      <c r="AU56" s="67"/>
-      <c r="AV56" s="66" t="s">
+      <c r="AU56" s="61"/>
+      <c r="AV56" s="60" t="s">
         <v>46</v>
       </c>
-      <c r="AW56" s="67"/>
-      <c r="AX56" s="66" t="s">
+      <c r="AW56" s="61"/>
+      <c r="AX56" s="60" t="s">
         <v>46</v>
       </c>
       <c r="AY56" s="68"/>
@@ -5277,16 +5277,16 @@
       <c r="AM60" s="28"/>
       <c r="AN60" s="28"/>
       <c r="AO60" s="28"/>
-      <c r="AP60" s="62"/>
-      <c r="AQ60" s="63"/>
-      <c r="AR60" s="64"/>
-      <c r="AS60" s="65"/>
-      <c r="AT60" s="62"/>
-      <c r="AU60" s="63"/>
-      <c r="AV60" s="64"/>
-      <c r="AW60" s="65"/>
-      <c r="AX60" s="62"/>
-      <c r="AY60" s="63"/>
+      <c r="AP60" s="66"/>
+      <c r="AQ60" s="67"/>
+      <c r="AR60" s="62"/>
+      <c r="AS60" s="63"/>
+      <c r="AT60" s="66"/>
+      <c r="AU60" s="67"/>
+      <c r="AV60" s="62"/>
+      <c r="AW60" s="63"/>
+      <c r="AX60" s="66"/>
+      <c r="AY60" s="67"/>
       <c r="AZ60" s="29">
         <v>0</v>
       </c>
@@ -5418,26 +5418,26 @@
       <c r="AM62" s="23"/>
       <c r="AN62" s="23"/>
       <c r="AO62" s="32"/>
-      <c r="AP62" s="60" t="s">
+      <c r="AP62" s="70" t="s">
         <v>44</v>
       </c>
-      <c r="AQ62" s="61"/>
-      <c r="AR62" s="60" t="s">
+      <c r="AQ62" s="71"/>
+      <c r="AR62" s="70" t="s">
         <v>44</v>
       </c>
-      <c r="AS62" s="61"/>
-      <c r="AT62" s="60" t="s">
+      <c r="AS62" s="71"/>
+      <c r="AT62" s="70" t="s">
         <v>44</v>
       </c>
-      <c r="AU62" s="61"/>
-      <c r="AV62" s="60" t="s">
+      <c r="AU62" s="71"/>
+      <c r="AV62" s="70" t="s">
         <v>44</v>
       </c>
-      <c r="AW62" s="61"/>
-      <c r="AX62" s="60" t="s">
+      <c r="AW62" s="71"/>
+      <c r="AX62" s="70" t="s">
         <v>44</v>
       </c>
-      <c r="AY62" s="69"/>
+      <c r="AY62" s="72"/>
       <c r="AZ62" s="33"/>
       <c r="BA62" s="24"/>
       <c r="BB62" s="24"/>
@@ -5514,26 +5514,26 @@
       <c r="AM66" s="28"/>
       <c r="AN66" s="28"/>
       <c r="AO66" s="28"/>
-      <c r="AP66" s="62">
+      <c r="AP66" s="66">
         <v>7.5</v>
       </c>
-      <c r="AQ66" s="63"/>
-      <c r="AR66" s="64">
+      <c r="AQ66" s="67"/>
+      <c r="AR66" s="62">
         <v>7.5</v>
       </c>
-      <c r="AS66" s="65"/>
-      <c r="AT66" s="62">
+      <c r="AS66" s="63"/>
+      <c r="AT66" s="66">
         <v>7.5</v>
       </c>
-      <c r="AU66" s="63"/>
-      <c r="AV66" s="64">
+      <c r="AU66" s="67"/>
+      <c r="AV66" s="62">
         <v>7.5</v>
       </c>
-      <c r="AW66" s="65"/>
-      <c r="AX66" s="62">
+      <c r="AW66" s="63"/>
+      <c r="AX66" s="66">
         <v>7.5</v>
       </c>
-      <c r="AY66" s="63"/>
+      <c r="AY66" s="67"/>
       <c r="AZ66" s="29">
         <v>0</v>
       </c>
@@ -5665,26 +5665,26 @@
       <c r="AM68" s="23"/>
       <c r="AN68" s="23"/>
       <c r="AO68" s="32"/>
-      <c r="AP68" s="66" t="s">
+      <c r="AP68" s="60" t="s">
         <v>46</v>
       </c>
-      <c r="AQ68" s="67"/>
-      <c r="AR68" s="66" t="s">
+      <c r="AQ68" s="61"/>
+      <c r="AR68" s="60" t="s">
         <v>46</v>
       </c>
-      <c r="AS68" s="67"/>
-      <c r="AT68" s="70" t="s">
+      <c r="AS68" s="61"/>
+      <c r="AT68" s="64" t="s">
         <v>45</v>
       </c>
-      <c r="AU68" s="71"/>
-      <c r="AV68" s="66" t="s">
+      <c r="AU68" s="69"/>
+      <c r="AV68" s="60" t="s">
         <v>46</v>
       </c>
-      <c r="AW68" s="67"/>
-      <c r="AX68" s="70" t="s">
+      <c r="AW68" s="61"/>
+      <c r="AX68" s="64" t="s">
         <v>45</v>
       </c>
-      <c r="AY68" s="72"/>
+      <c r="AY68" s="65"/>
       <c r="AZ68" s="33"/>
       <c r="BA68" s="24"/>
       <c r="BB68" s="24"/>
@@ -5761,26 +5761,26 @@
       <c r="AM72" s="28"/>
       <c r="AN72" s="28"/>
       <c r="AO72" s="28"/>
-      <c r="AP72" s="62">
+      <c r="AP72" s="66">
         <v>7.5</v>
       </c>
-      <c r="AQ72" s="63"/>
-      <c r="AR72" s="64">
+      <c r="AQ72" s="67"/>
+      <c r="AR72" s="62">
         <v>7.5</v>
       </c>
-      <c r="AS72" s="65"/>
-      <c r="AT72" s="62">
+      <c r="AS72" s="63"/>
+      <c r="AT72" s="66">
         <v>7.5</v>
       </c>
-      <c r="AU72" s="63"/>
-      <c r="AV72" s="64">
+      <c r="AU72" s="67"/>
+      <c r="AV72" s="62">
         <v>7.5</v>
       </c>
-      <c r="AW72" s="65"/>
-      <c r="AX72" s="62">
+      <c r="AW72" s="63"/>
+      <c r="AX72" s="66">
         <v>5</v>
       </c>
-      <c r="AY72" s="63"/>
+      <c r="AY72" s="67"/>
       <c r="AZ72" s="29">
         <v>0</v>
       </c>
@@ -5912,23 +5912,23 @@
       <c r="AM74" s="23"/>
       <c r="AN74" s="23"/>
       <c r="AO74" s="32"/>
-      <c r="AP74" s="66" t="s">
+      <c r="AP74" s="60" t="s">
         <v>46</v>
       </c>
-      <c r="AQ74" s="67"/>
-      <c r="AR74" s="66" t="s">
+      <c r="AQ74" s="61"/>
+      <c r="AR74" s="60" t="s">
         <v>46</v>
       </c>
-      <c r="AS74" s="67"/>
-      <c r="AT74" s="66" t="s">
+      <c r="AS74" s="61"/>
+      <c r="AT74" s="60" t="s">
         <v>46</v>
       </c>
-      <c r="AU74" s="67"/>
-      <c r="AV74" s="66" t="s">
+      <c r="AU74" s="61"/>
+      <c r="AV74" s="60" t="s">
         <v>46</v>
       </c>
-      <c r="AW74" s="67"/>
-      <c r="AX74" s="66" t="s">
+      <c r="AW74" s="61"/>
+      <c r="AX74" s="60" t="s">
         <v>46</v>
       </c>
       <c r="AY74" s="68"/>
@@ -6048,26 +6048,26 @@
       <c r="AM82" s="28"/>
       <c r="AN82" s="28"/>
       <c r="AO82" s="28"/>
-      <c r="AP82" s="62">
+      <c r="AP82" s="66">
         <v>7.5</v>
       </c>
-      <c r="AQ82" s="63"/>
-      <c r="AR82" s="64">
+      <c r="AQ82" s="67"/>
+      <c r="AR82" s="62">
         <v>7.5</v>
       </c>
-      <c r="AS82" s="65"/>
-      <c r="AT82" s="62">
+      <c r="AS82" s="63"/>
+      <c r="AT82" s="66">
         <v>7.5</v>
       </c>
-      <c r="AU82" s="63"/>
-      <c r="AV82" s="64">
+      <c r="AU82" s="67"/>
+      <c r="AV82" s="62">
         <v>7.5</v>
       </c>
-      <c r="AW82" s="65"/>
-      <c r="AX82" s="62">
+      <c r="AW82" s="63"/>
+      <c r="AX82" s="66">
         <v>5</v>
       </c>
-      <c r="AY82" s="63"/>
+      <c r="AY82" s="67"/>
       <c r="AZ82" s="29">
         <v>0</v>
       </c>
@@ -6199,23 +6199,23 @@
       <c r="AM84" s="23"/>
       <c r="AN84" s="23"/>
       <c r="AO84" s="32"/>
-      <c r="AP84" s="66" t="s">
+      <c r="AP84" s="60" t="s">
         <v>46</v>
       </c>
-      <c r="AQ84" s="67"/>
-      <c r="AR84" s="70" t="s">
+      <c r="AQ84" s="61"/>
+      <c r="AR84" s="64" t="s">
         <v>45</v>
       </c>
-      <c r="AS84" s="71"/>
-      <c r="AT84" s="66" t="s">
+      <c r="AS84" s="69"/>
+      <c r="AT84" s="60" t="s">
         <v>46</v>
       </c>
-      <c r="AU84" s="67"/>
-      <c r="AV84" s="66" t="s">
+      <c r="AU84" s="61"/>
+      <c r="AV84" s="60" t="s">
         <v>46</v>
       </c>
-      <c r="AW84" s="67"/>
-      <c r="AX84" s="66" t="s">
+      <c r="AW84" s="61"/>
+      <c r="AX84" s="60" t="s">
         <v>46</v>
       </c>
       <c r="AY84" s="68"/>
@@ -6298,26 +6298,26 @@
       <c r="AM88" s="28"/>
       <c r="AN88" s="28"/>
       <c r="AO88" s="28"/>
-      <c r="AP88" s="62">
+      <c r="AP88" s="66">
         <v>7.5</v>
       </c>
-      <c r="AQ88" s="63"/>
-      <c r="AR88" s="64">
+      <c r="AQ88" s="67"/>
+      <c r="AR88" s="62">
         <v>7.5</v>
       </c>
-      <c r="AS88" s="65"/>
-      <c r="AT88" s="62">
+      <c r="AS88" s="63"/>
+      <c r="AT88" s="66">
         <v>7.5</v>
       </c>
-      <c r="AU88" s="63"/>
-      <c r="AV88" s="64">
+      <c r="AU88" s="67"/>
+      <c r="AV88" s="62">
         <v>7.5</v>
       </c>
-      <c r="AW88" s="65"/>
-      <c r="AX88" s="62">
+      <c r="AW88" s="63"/>
+      <c r="AX88" s="66">
         <v>5</v>
       </c>
-      <c r="AY88" s="63"/>
+      <c r="AY88" s="67"/>
       <c r="AZ88" s="29">
         <v>0</v>
       </c>
@@ -6449,23 +6449,23 @@
       <c r="AM90" s="23"/>
       <c r="AN90" s="23"/>
       <c r="AO90" s="32"/>
-      <c r="AP90" s="66" t="s">
+      <c r="AP90" s="60" t="s">
         <v>46</v>
       </c>
-      <c r="AQ90" s="67"/>
-      <c r="AR90" s="66" t="s">
+      <c r="AQ90" s="61"/>
+      <c r="AR90" s="60" t="s">
         <v>46</v>
       </c>
-      <c r="AS90" s="67"/>
-      <c r="AT90" s="66" t="s">
+      <c r="AS90" s="61"/>
+      <c r="AT90" s="60" t="s">
         <v>46</v>
       </c>
-      <c r="AU90" s="67"/>
-      <c r="AV90" s="66" t="s">
+      <c r="AU90" s="61"/>
+      <c r="AV90" s="60" t="s">
         <v>46</v>
       </c>
-      <c r="AW90" s="67"/>
-      <c r="AX90" s="66" t="s">
+      <c r="AW90" s="61"/>
+      <c r="AX90" s="60" t="s">
         <v>46</v>
       </c>
       <c r="AY90" s="68"/>
@@ -6551,24 +6551,24 @@
       <c r="AM94" s="28"/>
       <c r="AN94" s="28"/>
       <c r="AO94" s="28"/>
-      <c r="AP94" s="62">
+      <c r="AP94" s="66">
         <v>7</v>
       </c>
-      <c r="AQ94" s="63"/>
-      <c r="AR94" s="64">
+      <c r="AQ94" s="67"/>
+      <c r="AR94" s="62">
         <v>7</v>
       </c>
-      <c r="AS94" s="65"/>
-      <c r="AT94" s="62">
+      <c r="AS94" s="63"/>
+      <c r="AT94" s="66">
         <v>7</v>
       </c>
-      <c r="AU94" s="63"/>
-      <c r="AV94" s="64">
+      <c r="AU94" s="67"/>
+      <c r="AV94" s="62">
         <v>7</v>
       </c>
-      <c r="AW94" s="65"/>
-      <c r="AX94" s="62"/>
-      <c r="AY94" s="63"/>
+      <c r="AW94" s="63"/>
+      <c r="AX94" s="66"/>
+      <c r="AY94" s="67"/>
       <c r="AZ94" s="29">
         <v>0</v>
       </c>
@@ -6700,26 +6700,26 @@
       <c r="AM96" s="23"/>
       <c r="AN96" s="23"/>
       <c r="AO96" s="32"/>
-      <c r="AP96" s="66" t="s">
+      <c r="AP96" s="60" t="s">
         <v>46</v>
       </c>
-      <c r="AQ96" s="67"/>
-      <c r="AR96" s="66" t="s">
+      <c r="AQ96" s="61"/>
+      <c r="AR96" s="60" t="s">
         <v>46</v>
       </c>
-      <c r="AS96" s="67"/>
-      <c r="AT96" s="66" t="s">
+      <c r="AS96" s="61"/>
+      <c r="AT96" s="60" t="s">
         <v>46</v>
       </c>
-      <c r="AU96" s="67"/>
-      <c r="AV96" s="66" t="s">
+      <c r="AU96" s="61"/>
+      <c r="AV96" s="60" t="s">
         <v>46</v>
       </c>
-      <c r="AW96" s="67"/>
-      <c r="AX96" s="60" t="s">
+      <c r="AW96" s="61"/>
+      <c r="AX96" s="70" t="s">
         <v>44</v>
       </c>
-      <c r="AY96" s="69"/>
+      <c r="AY96" s="72"/>
       <c r="AZ96" s="33"/>
       <c r="BA96" s="24"/>
       <c r="BB96" s="24"/>
@@ -6850,26 +6850,26 @@
       <c r="AM104" s="28"/>
       <c r="AN104" s="28"/>
       <c r="AO104" s="28"/>
-      <c r="AP104" s="62">
+      <c r="AP104" s="66">
         <v>7.5</v>
       </c>
-      <c r="AQ104" s="63"/>
-      <c r="AR104" s="64">
+      <c r="AQ104" s="67"/>
+      <c r="AR104" s="62">
         <v>7.5</v>
       </c>
-      <c r="AS104" s="65"/>
-      <c r="AT104" s="62">
+      <c r="AS104" s="63"/>
+      <c r="AT104" s="66">
         <v>7.5</v>
       </c>
-      <c r="AU104" s="63"/>
-      <c r="AV104" s="64">
+      <c r="AU104" s="67"/>
+      <c r="AV104" s="62">
         <v>9.5</v>
       </c>
-      <c r="AW104" s="65"/>
-      <c r="AX104" s="62">
+      <c r="AW104" s="63"/>
+      <c r="AX104" s="66">
         <v>5.5</v>
       </c>
-      <c r="AY104" s="63"/>
+      <c r="AY104" s="67"/>
       <c r="AZ104" s="29">
         <v>0</v>
       </c>
@@ -7004,23 +7004,23 @@
       <c r="AM106" s="23"/>
       <c r="AN106" s="23"/>
       <c r="AO106" s="32"/>
-      <c r="AP106" s="66" t="s">
+      <c r="AP106" s="60" t="s">
         <v>46</v>
       </c>
-      <c r="AQ106" s="67"/>
-      <c r="AR106" s="66" t="s">
+      <c r="AQ106" s="61"/>
+      <c r="AR106" s="60" t="s">
         <v>46</v>
       </c>
-      <c r="AS106" s="67"/>
-      <c r="AT106" s="66" t="s">
+      <c r="AS106" s="61"/>
+      <c r="AT106" s="60" t="s">
         <v>46</v>
       </c>
-      <c r="AU106" s="67"/>
-      <c r="AV106" s="66" t="s">
+      <c r="AU106" s="61"/>
+      <c r="AV106" s="60" t="s">
         <v>46</v>
       </c>
-      <c r="AW106" s="67"/>
-      <c r="AX106" s="66" t="s">
+      <c r="AW106" s="61"/>
+      <c r="AX106" s="60" t="s">
         <v>46</v>
       </c>
       <c r="AY106" s="68"/>
@@ -7146,26 +7146,26 @@
       <c r="AM113" s="28"/>
       <c r="AN113" s="28"/>
       <c r="AO113" s="28"/>
-      <c r="AP113" s="62">
+      <c r="AP113" s="66">
         <v>7.5</v>
       </c>
-      <c r="AQ113" s="63"/>
-      <c r="AR113" s="64">
+      <c r="AQ113" s="67"/>
+      <c r="AR113" s="62">
         <v>7.5</v>
       </c>
-      <c r="AS113" s="65"/>
-      <c r="AT113" s="62">
+      <c r="AS113" s="63"/>
+      <c r="AT113" s="66">
         <v>7.5</v>
       </c>
-      <c r="AU113" s="63"/>
-      <c r="AV113" s="64">
+      <c r="AU113" s="67"/>
+      <c r="AV113" s="62">
         <v>7.5</v>
       </c>
-      <c r="AW113" s="65"/>
-      <c r="AX113" s="62">
+      <c r="AW113" s="63"/>
+      <c r="AX113" s="66">
         <v>5</v>
       </c>
-      <c r="AY113" s="63"/>
+      <c r="AY113" s="67"/>
       <c r="AZ113" s="29">
         <v>0</v>
       </c>
@@ -7297,23 +7297,23 @@
       <c r="AM115" s="23"/>
       <c r="AN115" s="23"/>
       <c r="AO115" s="32"/>
-      <c r="AP115" s="66" t="s">
+      <c r="AP115" s="60" t="s">
         <v>46</v>
       </c>
-      <c r="AQ115" s="67"/>
-      <c r="AR115" s="66" t="s">
+      <c r="AQ115" s="61"/>
+      <c r="AR115" s="60" t="s">
         <v>46</v>
       </c>
-      <c r="AS115" s="67"/>
-      <c r="AT115" s="70" t="s">
+      <c r="AS115" s="61"/>
+      <c r="AT115" s="64" t="s">
         <v>45</v>
       </c>
-      <c r="AU115" s="71"/>
-      <c r="AV115" s="66" t="s">
+      <c r="AU115" s="69"/>
+      <c r="AV115" s="60" t="s">
         <v>46</v>
       </c>
-      <c r="AW115" s="67"/>
-      <c r="AX115" s="66" t="s">
+      <c r="AW115" s="61"/>
+      <c r="AX115" s="60" t="s">
         <v>46</v>
       </c>
       <c r="AY115" s="68"/>
@@ -7439,26 +7439,26 @@
       <c r="AM122" s="28"/>
       <c r="AN122" s="28"/>
       <c r="AO122" s="28"/>
-      <c r="AP122" s="62">
+      <c r="AP122" s="66">
         <v>7.5</v>
       </c>
-      <c r="AQ122" s="63"/>
-      <c r="AR122" s="64">
+      <c r="AQ122" s="67"/>
+      <c r="AR122" s="62">
         <v>7.5</v>
       </c>
-      <c r="AS122" s="65"/>
-      <c r="AT122" s="62">
+      <c r="AS122" s="63"/>
+      <c r="AT122" s="66">
         <v>7.5</v>
       </c>
-      <c r="AU122" s="63"/>
-      <c r="AV122" s="64">
+      <c r="AU122" s="67"/>
+      <c r="AV122" s="62">
         <v>7.5</v>
       </c>
-      <c r="AW122" s="65"/>
-      <c r="AX122" s="62">
+      <c r="AW122" s="63"/>
+      <c r="AX122" s="66">
         <v>5</v>
       </c>
-      <c r="AY122" s="63"/>
+      <c r="AY122" s="67"/>
       <c r="AZ122" s="29">
         <v>0</v>
       </c>
@@ -7590,23 +7590,23 @@
       <c r="AM124" s="23"/>
       <c r="AN124" s="23"/>
       <c r="AO124" s="32"/>
-      <c r="AP124" s="66" t="s">
+      <c r="AP124" s="60" t="s">
         <v>46</v>
       </c>
-      <c r="AQ124" s="67"/>
-      <c r="AR124" s="66" t="s">
+      <c r="AQ124" s="61"/>
+      <c r="AR124" s="60" t="s">
         <v>46</v>
       </c>
-      <c r="AS124" s="67"/>
-      <c r="AT124" s="66" t="s">
+      <c r="AS124" s="61"/>
+      <c r="AT124" s="60" t="s">
         <v>46</v>
       </c>
-      <c r="AU124" s="67"/>
-      <c r="AV124" s="66" t="s">
+      <c r="AU124" s="61"/>
+      <c r="AV124" s="60" t="s">
         <v>46</v>
       </c>
-      <c r="AW124" s="67"/>
-      <c r="AX124" s="66" t="s">
+      <c r="AW124" s="61"/>
+      <c r="AX124" s="60" t="s">
         <v>46</v>
       </c>
       <c r="AY124" s="68"/>
@@ -7686,26 +7686,26 @@
       <c r="AM128" s="28"/>
       <c r="AN128" s="28"/>
       <c r="AO128" s="28"/>
-      <c r="AP128" s="62">
+      <c r="AP128" s="66">
         <v>8.5</v>
       </c>
-      <c r="AQ128" s="63"/>
-      <c r="AR128" s="64">
+      <c r="AQ128" s="67"/>
+      <c r="AR128" s="62">
         <v>8.5</v>
       </c>
-      <c r="AS128" s="65"/>
-      <c r="AT128" s="62">
+      <c r="AS128" s="63"/>
+      <c r="AT128" s="66">
         <v>6.25</v>
       </c>
-      <c r="AU128" s="63"/>
-      <c r="AV128" s="64">
+      <c r="AU128" s="67"/>
+      <c r="AV128" s="62">
         <v>8.5</v>
       </c>
-      <c r="AW128" s="65"/>
-      <c r="AX128" s="62">
+      <c r="AW128" s="63"/>
+      <c r="AX128" s="66">
         <v>7.75</v>
       </c>
-      <c r="AY128" s="63"/>
+      <c r="AY128" s="67"/>
       <c r="AZ128" s="29">
         <v>0</v>
       </c>
@@ -7837,23 +7837,23 @@
       <c r="AM130" s="23"/>
       <c r="AN130" s="23"/>
       <c r="AO130" s="32"/>
-      <c r="AP130" s="66" t="s">
+      <c r="AP130" s="60" t="s">
         <v>46</v>
       </c>
-      <c r="AQ130" s="67"/>
-      <c r="AR130" s="66" t="s">
+      <c r="AQ130" s="61"/>
+      <c r="AR130" s="60" t="s">
         <v>46</v>
       </c>
-      <c r="AS130" s="67"/>
-      <c r="AT130" s="66" t="s">
+      <c r="AS130" s="61"/>
+      <c r="AT130" s="60" t="s">
         <v>46</v>
       </c>
-      <c r="AU130" s="67"/>
-      <c r="AV130" s="66" t="s">
+      <c r="AU130" s="61"/>
+      <c r="AV130" s="60" t="s">
         <v>46</v>
       </c>
-      <c r="AW130" s="67"/>
-      <c r="AX130" s="66" t="s">
+      <c r="AW130" s="61"/>
+      <c r="AX130" s="60" t="s">
         <v>46</v>
       </c>
       <c r="AY130" s="68"/>
@@ -7963,16 +7963,16 @@
       <c r="AM134" s="28"/>
       <c r="AN134" s="28"/>
       <c r="AO134" s="28"/>
-      <c r="AP134" s="62"/>
-      <c r="AQ134" s="63"/>
-      <c r="AR134" s="64"/>
-      <c r="AS134" s="65"/>
-      <c r="AT134" s="62"/>
-      <c r="AU134" s="63"/>
-      <c r="AV134" s="64"/>
-      <c r="AW134" s="65"/>
-      <c r="AX134" s="62"/>
-      <c r="AY134" s="63"/>
+      <c r="AP134" s="66"/>
+      <c r="AQ134" s="67"/>
+      <c r="AR134" s="62"/>
+      <c r="AS134" s="63"/>
+      <c r="AT134" s="66"/>
+      <c r="AU134" s="67"/>
+      <c r="AV134" s="62"/>
+      <c r="AW134" s="63"/>
+      <c r="AX134" s="66"/>
+      <c r="AY134" s="67"/>
       <c r="AZ134" s="29">
         <v>0</v>
       </c>
@@ -8104,26 +8104,26 @@
       <c r="AM136" s="23"/>
       <c r="AN136" s="23"/>
       <c r="AO136" s="32"/>
-      <c r="AP136" s="60" t="s">
+      <c r="AP136" s="70" t="s">
         <v>44</v>
       </c>
-      <c r="AQ136" s="61"/>
-      <c r="AR136" s="60" t="s">
+      <c r="AQ136" s="71"/>
+      <c r="AR136" s="70" t="s">
         <v>44</v>
       </c>
-      <c r="AS136" s="61"/>
-      <c r="AT136" s="60" t="s">
+      <c r="AS136" s="71"/>
+      <c r="AT136" s="70" t="s">
         <v>44</v>
       </c>
-      <c r="AU136" s="61"/>
-      <c r="AV136" s="60" t="s">
+      <c r="AU136" s="71"/>
+      <c r="AV136" s="70" t="s">
         <v>44</v>
       </c>
-      <c r="AW136" s="61"/>
-      <c r="AX136" s="60" t="s">
+      <c r="AW136" s="71"/>
+      <c r="AX136" s="70" t="s">
         <v>44</v>
       </c>
-      <c r="AY136" s="69"/>
+      <c r="AY136" s="72"/>
       <c r="AZ136" s="33"/>
       <c r="BA136" s="24"/>
       <c r="BB136" s="24"/>
@@ -8336,26 +8336,26 @@
       <c r="AM150" s="28"/>
       <c r="AN150" s="28"/>
       <c r="AO150" s="28"/>
-      <c r="AP150" s="62">
+      <c r="AP150" s="66">
         <v>7.5</v>
       </c>
-      <c r="AQ150" s="63"/>
-      <c r="AR150" s="64">
+      <c r="AQ150" s="67"/>
+      <c r="AR150" s="62">
         <v>7.5</v>
       </c>
-      <c r="AS150" s="65"/>
-      <c r="AT150" s="62">
+      <c r="AS150" s="63"/>
+      <c r="AT150" s="66">
         <v>7.5</v>
       </c>
-      <c r="AU150" s="63"/>
-      <c r="AV150" s="64">
+      <c r="AU150" s="67"/>
+      <c r="AV150" s="62">
         <v>7.5</v>
       </c>
-      <c r="AW150" s="65"/>
-      <c r="AX150" s="62">
+      <c r="AW150" s="63"/>
+      <c r="AX150" s="66">
         <v>6</v>
       </c>
-      <c r="AY150" s="63"/>
+      <c r="AY150" s="67"/>
       <c r="AZ150" s="29">
         <v>0</v>
       </c>
@@ -8490,23 +8490,23 @@
       <c r="AM152" s="23"/>
       <c r="AN152" s="23"/>
       <c r="AO152" s="32"/>
-      <c r="AP152" s="66" t="s">
+      <c r="AP152" s="60" t="s">
         <v>46</v>
       </c>
-      <c r="AQ152" s="67"/>
-      <c r="AR152" s="66" t="s">
+      <c r="AQ152" s="61"/>
+      <c r="AR152" s="60" t="s">
         <v>46</v>
       </c>
-      <c r="AS152" s="67"/>
-      <c r="AT152" s="66" t="s">
+      <c r="AS152" s="61"/>
+      <c r="AT152" s="60" t="s">
         <v>46</v>
       </c>
-      <c r="AU152" s="67"/>
-      <c r="AV152" s="66" t="s">
+      <c r="AU152" s="61"/>
+      <c r="AV152" s="60" t="s">
         <v>46</v>
       </c>
-      <c r="AW152" s="67"/>
-      <c r="AX152" s="66" t="s">
+      <c r="AW152" s="61"/>
+      <c r="AX152" s="60" t="s">
         <v>46</v>
       </c>
       <c r="AY152" s="68"/>
@@ -8518,18 +8518,186 @@
   </sheetData>
   <dataConsolidate/>
   <mergeCells count="212">
-    <mergeCell ref="AR1:AS1"/>
-    <mergeCell ref="AT1:AU1"/>
-    <mergeCell ref="AV1:AW1"/>
-    <mergeCell ref="AX1:AY1"/>
-    <mergeCell ref="AZ1:BA1"/>
-    <mergeCell ref="BB1:BC1"/>
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="C1:C2"/>
-    <mergeCell ref="D1:D2"/>
-    <mergeCell ref="E1:Y1"/>
-    <mergeCell ref="Z1:AO1"/>
-    <mergeCell ref="AP1:AQ1"/>
+    <mergeCell ref="AP136:AQ136"/>
+    <mergeCell ref="AP134:AQ134"/>
+    <mergeCell ref="AR136:AS136"/>
+    <mergeCell ref="AR134:AS134"/>
+    <mergeCell ref="AT136:AU136"/>
+    <mergeCell ref="AT134:AU134"/>
+    <mergeCell ref="AV152:AW152"/>
+    <mergeCell ref="AV150:AW150"/>
+    <mergeCell ref="AX152:AY152"/>
+    <mergeCell ref="AX150:AY150"/>
+    <mergeCell ref="AV136:AW136"/>
+    <mergeCell ref="AV134:AW134"/>
+    <mergeCell ref="AX136:AY136"/>
+    <mergeCell ref="AX134:AY134"/>
+    <mergeCell ref="AP152:AQ152"/>
+    <mergeCell ref="AP150:AQ150"/>
+    <mergeCell ref="AR152:AS152"/>
+    <mergeCell ref="AR150:AS150"/>
+    <mergeCell ref="AT152:AU152"/>
+    <mergeCell ref="AT150:AU150"/>
+    <mergeCell ref="AP130:AQ130"/>
+    <mergeCell ref="AP128:AQ128"/>
+    <mergeCell ref="AR130:AS130"/>
+    <mergeCell ref="AR128:AS128"/>
+    <mergeCell ref="AT130:AU130"/>
+    <mergeCell ref="AT128:AU128"/>
+    <mergeCell ref="AV130:AW130"/>
+    <mergeCell ref="AV128:AW128"/>
+    <mergeCell ref="AX130:AY130"/>
+    <mergeCell ref="AX128:AY128"/>
+    <mergeCell ref="AP124:AQ124"/>
+    <mergeCell ref="AP122:AQ122"/>
+    <mergeCell ref="AR124:AS124"/>
+    <mergeCell ref="AR122:AS122"/>
+    <mergeCell ref="AT124:AU124"/>
+    <mergeCell ref="AT122:AU122"/>
+    <mergeCell ref="AV124:AW124"/>
+    <mergeCell ref="AV122:AW122"/>
+    <mergeCell ref="AX124:AY124"/>
+    <mergeCell ref="AX122:AY122"/>
+    <mergeCell ref="AP115:AQ115"/>
+    <mergeCell ref="AP113:AQ113"/>
+    <mergeCell ref="AR115:AS115"/>
+    <mergeCell ref="AR113:AS113"/>
+    <mergeCell ref="AT115:AU115"/>
+    <mergeCell ref="AT113:AU113"/>
+    <mergeCell ref="AV115:AW115"/>
+    <mergeCell ref="AV113:AW113"/>
+    <mergeCell ref="AX115:AY115"/>
+    <mergeCell ref="AX113:AY113"/>
+    <mergeCell ref="AP106:AQ106"/>
+    <mergeCell ref="AP104:AQ104"/>
+    <mergeCell ref="AR106:AS106"/>
+    <mergeCell ref="AR104:AS104"/>
+    <mergeCell ref="AT106:AU106"/>
+    <mergeCell ref="AT104:AU104"/>
+    <mergeCell ref="AV106:AW106"/>
+    <mergeCell ref="AV104:AW104"/>
+    <mergeCell ref="AX106:AY106"/>
+    <mergeCell ref="AX104:AY104"/>
+    <mergeCell ref="AP96:AQ96"/>
+    <mergeCell ref="AP94:AQ94"/>
+    <mergeCell ref="AR96:AS96"/>
+    <mergeCell ref="AR94:AS94"/>
+    <mergeCell ref="AT96:AU96"/>
+    <mergeCell ref="AT94:AU94"/>
+    <mergeCell ref="AV96:AW96"/>
+    <mergeCell ref="AV94:AW94"/>
+    <mergeCell ref="AX96:AY96"/>
+    <mergeCell ref="AX94:AY94"/>
+    <mergeCell ref="AP90:AQ90"/>
+    <mergeCell ref="AP88:AQ88"/>
+    <mergeCell ref="AR90:AS90"/>
+    <mergeCell ref="AR88:AS88"/>
+    <mergeCell ref="AT90:AU90"/>
+    <mergeCell ref="AT88:AU88"/>
+    <mergeCell ref="AV90:AW90"/>
+    <mergeCell ref="AV88:AW88"/>
+    <mergeCell ref="AX90:AY90"/>
+    <mergeCell ref="AX88:AY88"/>
+    <mergeCell ref="AP84:AQ84"/>
+    <mergeCell ref="AP82:AQ82"/>
+    <mergeCell ref="AR84:AS84"/>
+    <mergeCell ref="AR82:AS82"/>
+    <mergeCell ref="AT84:AU84"/>
+    <mergeCell ref="AT82:AU82"/>
+    <mergeCell ref="AV84:AW84"/>
+    <mergeCell ref="AV82:AW82"/>
+    <mergeCell ref="AX84:AY84"/>
+    <mergeCell ref="AX82:AY82"/>
+    <mergeCell ref="AP74:AQ74"/>
+    <mergeCell ref="AP72:AQ72"/>
+    <mergeCell ref="AR74:AS74"/>
+    <mergeCell ref="AR72:AS72"/>
+    <mergeCell ref="AT74:AU74"/>
+    <mergeCell ref="AT72:AU72"/>
+    <mergeCell ref="AV74:AW74"/>
+    <mergeCell ref="AV72:AW72"/>
+    <mergeCell ref="AX74:AY74"/>
+    <mergeCell ref="AX72:AY72"/>
+    <mergeCell ref="AP68:AQ68"/>
+    <mergeCell ref="AP66:AQ66"/>
+    <mergeCell ref="AR68:AS68"/>
+    <mergeCell ref="AR66:AS66"/>
+    <mergeCell ref="AT68:AU68"/>
+    <mergeCell ref="AT66:AU66"/>
+    <mergeCell ref="AV68:AW68"/>
+    <mergeCell ref="AV66:AW66"/>
+    <mergeCell ref="AX68:AY68"/>
+    <mergeCell ref="AX66:AY66"/>
+    <mergeCell ref="AP62:AQ62"/>
+    <mergeCell ref="AP60:AQ60"/>
+    <mergeCell ref="AR62:AS62"/>
+    <mergeCell ref="AR60:AS60"/>
+    <mergeCell ref="AT62:AU62"/>
+    <mergeCell ref="AT60:AU60"/>
+    <mergeCell ref="AV62:AW62"/>
+    <mergeCell ref="AV60:AW60"/>
+    <mergeCell ref="AX62:AY62"/>
+    <mergeCell ref="AX60:AY60"/>
+    <mergeCell ref="AP56:AQ56"/>
+    <mergeCell ref="AP54:AQ54"/>
+    <mergeCell ref="AR56:AS56"/>
+    <mergeCell ref="AR54:AS54"/>
+    <mergeCell ref="AT56:AU56"/>
+    <mergeCell ref="AT54:AU54"/>
+    <mergeCell ref="AV56:AW56"/>
+    <mergeCell ref="AV54:AW54"/>
+    <mergeCell ref="AX56:AY56"/>
+    <mergeCell ref="AX54:AY54"/>
+    <mergeCell ref="AP50:AQ50"/>
+    <mergeCell ref="AP48:AQ48"/>
+    <mergeCell ref="AR50:AS50"/>
+    <mergeCell ref="AR48:AS48"/>
+    <mergeCell ref="AT50:AU50"/>
+    <mergeCell ref="AT48:AU48"/>
+    <mergeCell ref="AV50:AW50"/>
+    <mergeCell ref="AV48:AW48"/>
+    <mergeCell ref="AX50:AY50"/>
+    <mergeCell ref="AX48:AY48"/>
+    <mergeCell ref="AP43:AQ43"/>
+    <mergeCell ref="AP41:AQ41"/>
+    <mergeCell ref="AR43:AS43"/>
+    <mergeCell ref="AR41:AS41"/>
+    <mergeCell ref="AT43:AU43"/>
+    <mergeCell ref="AT41:AU41"/>
+    <mergeCell ref="AV43:AW43"/>
+    <mergeCell ref="AV41:AW41"/>
+    <mergeCell ref="AX43:AY43"/>
+    <mergeCell ref="AX41:AY41"/>
+    <mergeCell ref="AP37:AQ37"/>
+    <mergeCell ref="AP35:AQ35"/>
+    <mergeCell ref="AR37:AS37"/>
+    <mergeCell ref="AR35:AS35"/>
+    <mergeCell ref="AT37:AU37"/>
+    <mergeCell ref="AT35:AU35"/>
+    <mergeCell ref="AV37:AW37"/>
+    <mergeCell ref="AV35:AW35"/>
+    <mergeCell ref="AX37:AY37"/>
+    <mergeCell ref="AX35:AY35"/>
+    <mergeCell ref="AP31:AQ31"/>
+    <mergeCell ref="AP29:AQ29"/>
+    <mergeCell ref="AR31:AS31"/>
+    <mergeCell ref="AR29:AS29"/>
+    <mergeCell ref="AT31:AU31"/>
+    <mergeCell ref="AT29:AU29"/>
+    <mergeCell ref="AV31:AW31"/>
+    <mergeCell ref="AV29:AW29"/>
+    <mergeCell ref="AX31:AY31"/>
+    <mergeCell ref="AX29:AY29"/>
+    <mergeCell ref="AP25:AQ25"/>
+    <mergeCell ref="AP23:AQ23"/>
+    <mergeCell ref="AR25:AS25"/>
+    <mergeCell ref="AR23:AS23"/>
+    <mergeCell ref="AT25:AU25"/>
+    <mergeCell ref="AT23:AU23"/>
+    <mergeCell ref="AV25:AW25"/>
+    <mergeCell ref="AV23:AW23"/>
+    <mergeCell ref="AX25:AY25"/>
+    <mergeCell ref="AX23:AY23"/>
     <mergeCell ref="AV10:AW10"/>
     <mergeCell ref="AV8:AW8"/>
     <mergeCell ref="AX10:AY10"/>
@@ -8550,186 +8718,18 @@
     <mergeCell ref="AV17:AW17"/>
     <mergeCell ref="AX19:AY19"/>
     <mergeCell ref="AX17:AY17"/>
-    <mergeCell ref="AP25:AQ25"/>
-    <mergeCell ref="AP23:AQ23"/>
-    <mergeCell ref="AR25:AS25"/>
-    <mergeCell ref="AR23:AS23"/>
-    <mergeCell ref="AT25:AU25"/>
-    <mergeCell ref="AT23:AU23"/>
-    <mergeCell ref="AV25:AW25"/>
-    <mergeCell ref="AV23:AW23"/>
-    <mergeCell ref="AX25:AY25"/>
-    <mergeCell ref="AX23:AY23"/>
-    <mergeCell ref="AP31:AQ31"/>
-    <mergeCell ref="AP29:AQ29"/>
-    <mergeCell ref="AR31:AS31"/>
-    <mergeCell ref="AR29:AS29"/>
-    <mergeCell ref="AT31:AU31"/>
-    <mergeCell ref="AT29:AU29"/>
-    <mergeCell ref="AV31:AW31"/>
-    <mergeCell ref="AV29:AW29"/>
-    <mergeCell ref="AX31:AY31"/>
-    <mergeCell ref="AX29:AY29"/>
-    <mergeCell ref="AP37:AQ37"/>
-    <mergeCell ref="AP35:AQ35"/>
-    <mergeCell ref="AR37:AS37"/>
-    <mergeCell ref="AR35:AS35"/>
-    <mergeCell ref="AT37:AU37"/>
-    <mergeCell ref="AT35:AU35"/>
-    <mergeCell ref="AV37:AW37"/>
-    <mergeCell ref="AV35:AW35"/>
-    <mergeCell ref="AX37:AY37"/>
-    <mergeCell ref="AX35:AY35"/>
-    <mergeCell ref="AP43:AQ43"/>
-    <mergeCell ref="AP41:AQ41"/>
-    <mergeCell ref="AR43:AS43"/>
-    <mergeCell ref="AR41:AS41"/>
-    <mergeCell ref="AT43:AU43"/>
-    <mergeCell ref="AT41:AU41"/>
-    <mergeCell ref="AV43:AW43"/>
-    <mergeCell ref="AV41:AW41"/>
-    <mergeCell ref="AX43:AY43"/>
-    <mergeCell ref="AX41:AY41"/>
-    <mergeCell ref="AP50:AQ50"/>
-    <mergeCell ref="AP48:AQ48"/>
-    <mergeCell ref="AR50:AS50"/>
-    <mergeCell ref="AR48:AS48"/>
-    <mergeCell ref="AT50:AU50"/>
-    <mergeCell ref="AT48:AU48"/>
-    <mergeCell ref="AV50:AW50"/>
-    <mergeCell ref="AV48:AW48"/>
-    <mergeCell ref="AX50:AY50"/>
-    <mergeCell ref="AX48:AY48"/>
-    <mergeCell ref="AP56:AQ56"/>
-    <mergeCell ref="AP54:AQ54"/>
-    <mergeCell ref="AR56:AS56"/>
-    <mergeCell ref="AR54:AS54"/>
-    <mergeCell ref="AT56:AU56"/>
-    <mergeCell ref="AT54:AU54"/>
-    <mergeCell ref="AV56:AW56"/>
-    <mergeCell ref="AV54:AW54"/>
-    <mergeCell ref="AX56:AY56"/>
-    <mergeCell ref="AX54:AY54"/>
-    <mergeCell ref="AP62:AQ62"/>
-    <mergeCell ref="AP60:AQ60"/>
-    <mergeCell ref="AR62:AS62"/>
-    <mergeCell ref="AR60:AS60"/>
-    <mergeCell ref="AT62:AU62"/>
-    <mergeCell ref="AT60:AU60"/>
-    <mergeCell ref="AV62:AW62"/>
-    <mergeCell ref="AV60:AW60"/>
-    <mergeCell ref="AX62:AY62"/>
-    <mergeCell ref="AX60:AY60"/>
-    <mergeCell ref="AP68:AQ68"/>
-    <mergeCell ref="AP66:AQ66"/>
-    <mergeCell ref="AR68:AS68"/>
-    <mergeCell ref="AR66:AS66"/>
-    <mergeCell ref="AT68:AU68"/>
-    <mergeCell ref="AT66:AU66"/>
-    <mergeCell ref="AV68:AW68"/>
-    <mergeCell ref="AV66:AW66"/>
-    <mergeCell ref="AX68:AY68"/>
-    <mergeCell ref="AX66:AY66"/>
-    <mergeCell ref="AP74:AQ74"/>
-    <mergeCell ref="AP72:AQ72"/>
-    <mergeCell ref="AR74:AS74"/>
-    <mergeCell ref="AR72:AS72"/>
-    <mergeCell ref="AT74:AU74"/>
-    <mergeCell ref="AT72:AU72"/>
-    <mergeCell ref="AV74:AW74"/>
-    <mergeCell ref="AV72:AW72"/>
-    <mergeCell ref="AX74:AY74"/>
-    <mergeCell ref="AX72:AY72"/>
-    <mergeCell ref="AP84:AQ84"/>
-    <mergeCell ref="AP82:AQ82"/>
-    <mergeCell ref="AR84:AS84"/>
-    <mergeCell ref="AR82:AS82"/>
-    <mergeCell ref="AT84:AU84"/>
-    <mergeCell ref="AT82:AU82"/>
-    <mergeCell ref="AV84:AW84"/>
-    <mergeCell ref="AV82:AW82"/>
-    <mergeCell ref="AX84:AY84"/>
-    <mergeCell ref="AX82:AY82"/>
-    <mergeCell ref="AP90:AQ90"/>
-    <mergeCell ref="AP88:AQ88"/>
-    <mergeCell ref="AR90:AS90"/>
-    <mergeCell ref="AR88:AS88"/>
-    <mergeCell ref="AT90:AU90"/>
-    <mergeCell ref="AT88:AU88"/>
-    <mergeCell ref="AV90:AW90"/>
-    <mergeCell ref="AV88:AW88"/>
-    <mergeCell ref="AX90:AY90"/>
-    <mergeCell ref="AX88:AY88"/>
-    <mergeCell ref="AP96:AQ96"/>
-    <mergeCell ref="AP94:AQ94"/>
-    <mergeCell ref="AR96:AS96"/>
-    <mergeCell ref="AR94:AS94"/>
-    <mergeCell ref="AT96:AU96"/>
-    <mergeCell ref="AT94:AU94"/>
-    <mergeCell ref="AV96:AW96"/>
-    <mergeCell ref="AV94:AW94"/>
-    <mergeCell ref="AX96:AY96"/>
-    <mergeCell ref="AX94:AY94"/>
-    <mergeCell ref="AP106:AQ106"/>
-    <mergeCell ref="AP104:AQ104"/>
-    <mergeCell ref="AR106:AS106"/>
-    <mergeCell ref="AR104:AS104"/>
-    <mergeCell ref="AT106:AU106"/>
-    <mergeCell ref="AT104:AU104"/>
-    <mergeCell ref="AV106:AW106"/>
-    <mergeCell ref="AV104:AW104"/>
-    <mergeCell ref="AX106:AY106"/>
-    <mergeCell ref="AX104:AY104"/>
-    <mergeCell ref="AP115:AQ115"/>
-    <mergeCell ref="AP113:AQ113"/>
-    <mergeCell ref="AR115:AS115"/>
-    <mergeCell ref="AR113:AS113"/>
-    <mergeCell ref="AT115:AU115"/>
-    <mergeCell ref="AT113:AU113"/>
-    <mergeCell ref="AV115:AW115"/>
-    <mergeCell ref="AV113:AW113"/>
-    <mergeCell ref="AX115:AY115"/>
-    <mergeCell ref="AX113:AY113"/>
-    <mergeCell ref="AP124:AQ124"/>
-    <mergeCell ref="AP122:AQ122"/>
-    <mergeCell ref="AR124:AS124"/>
-    <mergeCell ref="AR122:AS122"/>
-    <mergeCell ref="AT124:AU124"/>
-    <mergeCell ref="AT122:AU122"/>
-    <mergeCell ref="AV124:AW124"/>
-    <mergeCell ref="AV122:AW122"/>
-    <mergeCell ref="AX124:AY124"/>
-    <mergeCell ref="AX122:AY122"/>
-    <mergeCell ref="AP130:AQ130"/>
-    <mergeCell ref="AP128:AQ128"/>
-    <mergeCell ref="AR130:AS130"/>
-    <mergeCell ref="AR128:AS128"/>
-    <mergeCell ref="AT130:AU130"/>
-    <mergeCell ref="AT128:AU128"/>
-    <mergeCell ref="AV130:AW130"/>
-    <mergeCell ref="AV128:AW128"/>
-    <mergeCell ref="AX130:AY130"/>
-    <mergeCell ref="AX128:AY128"/>
-    <mergeCell ref="AP136:AQ136"/>
-    <mergeCell ref="AP134:AQ134"/>
-    <mergeCell ref="AR136:AS136"/>
-    <mergeCell ref="AR134:AS134"/>
-    <mergeCell ref="AT136:AU136"/>
-    <mergeCell ref="AT134:AU134"/>
-    <mergeCell ref="AV152:AW152"/>
-    <mergeCell ref="AV150:AW150"/>
-    <mergeCell ref="AX152:AY152"/>
-    <mergeCell ref="AX150:AY150"/>
-    <mergeCell ref="AV136:AW136"/>
-    <mergeCell ref="AV134:AW134"/>
-    <mergeCell ref="AX136:AY136"/>
-    <mergeCell ref="AX134:AY134"/>
-    <mergeCell ref="AP152:AQ152"/>
-    <mergeCell ref="AP150:AQ150"/>
-    <mergeCell ref="AR152:AS152"/>
-    <mergeCell ref="AR150:AS150"/>
-    <mergeCell ref="AT152:AU152"/>
-    <mergeCell ref="AT150:AU150"/>
+    <mergeCell ref="AR1:AS1"/>
+    <mergeCell ref="AT1:AU1"/>
+    <mergeCell ref="AV1:AW1"/>
+    <mergeCell ref="AX1:AY1"/>
+    <mergeCell ref="AZ1:BA1"/>
+    <mergeCell ref="BB1:BC1"/>
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="C1:C2"/>
+    <mergeCell ref="D1:D2"/>
+    <mergeCell ref="E1:Y1"/>
+    <mergeCell ref="Z1:AO1"/>
+    <mergeCell ref="AP1:AQ1"/>
   </mergeCells>
   <conditionalFormatting sqref="D10">
     <cfRule type="cellIs" dxfId="59" priority="59" operator="equal">

</xml_diff>